<commit_message>
need HOBO data from winter 2026
</commit_message>
<xml_diff>
--- a/data/adventure_mine.xlsx
+++ b/data/adventure_mine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michigantech-my.sharepoint.com/personal/tmbarnes_mtu_edu/Documents/PhD/HOBO/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_22929B9079AD8EF8208E6A1B326FA8FFE34C6004" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{837D47E5-9F50-1345-BA98-62B9E834FFD4}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="11_22929B9079AD8EF8208E6A1B326FA8FFE34C6004" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A149D809-D791-9D4C-A210-9D4020389C54}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34520" yWindow="1800" windowWidth="29400" windowHeight="16820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="overlook" sheetId="1" r:id="rId1"/>
@@ -36,18 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="91">
   <si>
     <t>#</t>
   </si>
   <si>
     <t>Date-Time (EST/EDT)</t>
-  </si>
-  <si>
-    <t>Adventure Temp , °C</t>
-  </si>
-  <si>
-    <t>Adventure Light , lux</t>
   </si>
   <si>
     <t>Host Connected</t>
@@ -284,12 +278,6 @@
     <t>.11</t>
   </si>
   <si>
-    <t>wet_bulb</t>
-  </si>
-  <si>
-    <t>dry_bulb</t>
-  </si>
-  <si>
     <t>mean humidity</t>
   </si>
   <si>
@@ -303,6 +291,24 @@
   </si>
   <si>
     <t>all temps from all loggers</t>
+  </si>
+  <si>
+    <t>probe</t>
+  </si>
+  <si>
+    <t>integrated</t>
+  </si>
+  <si>
+    <t>rh</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>temp</t>
+  </si>
+  <si>
+    <t>light</t>
   </si>
 </sst>
 </file>
@@ -354,7 +360,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -370,6 +376,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="C" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
@@ -727,23 +734,23 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
+      <c r="B1" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -7547,20 +7554,23 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" s="11" t="s">
+        <v>88</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>83</v>
+        <v>86</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>87</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -13139,13 +13149,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -13156,7 +13166,7 @@
         <v>45692.45888888889</v>
       </c>
       <c r="E2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -13167,10 +13177,10 @@
         <v>45756.558854166666</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -13192,393 +13202,393 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C4" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C5" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C7" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C8" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C9" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C10" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C11" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C12" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C14" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C15" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C16" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C17" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C18" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C19" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C20" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C21" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C22" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C23" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C24" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C25" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C26" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C27" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D27" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C28" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C29" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C32" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D32" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C33" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D33" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C35" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D35" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C36" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D36" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C37" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C38" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D38" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C39" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D39" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C40" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C41" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C44" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D44" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C45" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C47" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D47" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C48" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D48" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C49" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D49" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C50" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D50" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C51" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D51" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C52" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D52" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="53" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C53" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D53" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>